<commit_message>
xlstream-eval: fix statistical error types and PERCENTILE.EXC n=1
Revert percentile/quartile error types back to #NUM! (Excel agrees
with original code, LO cached wrong #VALUE!). Fix PERCENTILE.EXC
rejecting single-value arrays — lower==upper guard was too strict.
Fixtures Excel-recalculated.
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/statistical/quartile.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/statistical/quartile.xlsx
@@ -1,18 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-conformance/crates/xlstream-eval/tests/fixtures/statistical/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_85C7D3F3BC51D74835E711D805284C1BDCD4D4CD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="16380" windowHeight="8200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -23,56 +39,38 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
-    <t xml:space="preserve">Values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mixed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">skip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XS</t>
+    <t>Values</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Same</t>
+  </si>
+  <si>
+    <t>Mixed</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>skip</t>
+  </si>
+  <si>
+    <t>XS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -84,7 +82,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -92,50 +90,30 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -177,12 +155,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -211,7 +189,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -232,7 +210,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -283,7 +261,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -301,272 +279,258 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2">
         <v>10</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2">
         <v>7</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="G2" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, 0)</f>
+      <c r="G2">
+        <f>_xlfn.QUARTILE.INC(A2:A11, 0)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3">
         <v>20</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3">
         <v>7</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, 1)</f>
+      <c r="G3">
+        <f>_xlfn.QUARTILE.INC(A2:A11, 1)</f>
         <v>3.25</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4">
         <v>30</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4">
         <v>7</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4">
         <v>3</v>
       </c>
-      <c r="G4" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, 2)</f>
+      <c r="G4">
+        <f>_xlfn.QUARTILE.INC(A2:A11, 2)</f>
         <v>5.5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5">
         <v>7</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" t="s">
         <v>5</v>
       </c>
-      <c r="G5" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, 3)</f>
+      <c r="G5">
+        <f>_xlfn.QUARTILE.INC(A2:A11, 3)</f>
         <v>7.75</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>5</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6">
         <v>5</v>
       </c>
-      <c r="G6" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, 4)</f>
+      <c r="G6">
+        <f>_xlfn.QUARTILE.INC(A2:A11, 4)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>6</v>
       </c>
-      <c r="G7" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.EXC(A2:A11, 1)</f>
+      <c r="G7">
+        <f>_xlfn.QUARTILE.EXC(A2:A11, 1)</f>
         <v>2.75</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>7</v>
       </c>
-      <c r="G8" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.EXC(A2:A11, 2)</f>
+      <c r="G8">
+        <f>_xlfn.QUARTILE.EXC(A2:A11, 2)</f>
         <v>5.5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9">
         <v>8</v>
       </c>
-      <c r="G9" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.EXC(A2:A11, 3)</f>
+      <c r="G9">
+        <f>_xlfn.QUARTILE.EXC(A2:A11, 3)</f>
         <v>8.25</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10">
         <v>9</v>
       </c>
-      <c r="G10" s="0" t="e">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, 5)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="G10" t="e">
+        <f>_xlfn.QUARTILE.INC(A2:A11, 5)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11">
         <v>10</v>
       </c>
-      <c r="G11" s="0" t="e">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, -1)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G12" s="0" t="e">
-        <f aca="false">_xlfn.QUARTILE.EXC(A2:A11, 0)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G13" s="0" t="e">
-        <f aca="false">_xlfn.QUARTILE.EXC(A2:A11, 4)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G14" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(C2:C5, 2)</f>
+      <c r="G11" t="e">
+        <f>_xlfn.QUARTILE.INC(A2:A11, -1)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G12" t="e">
+        <f>_xlfn.QUARTILE.EXC(A2:A11, 0)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G13" t="e">
+        <f>_xlfn.QUARTILE.EXC(A2:A11, 4)</f>
+        <v>#NUM!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G14">
+        <f>_xlfn.QUARTILE.INC(C2:C5, 2)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G15" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(D2:D6, 2)</f>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G15">
+        <f>_xlfn.QUARTILE.INC(D2:D6, 2)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G16" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.EXC(D2:D6, 2)</f>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G16">
+        <f>_xlfn.QUARTILE.EXC(D2:D6, 2)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G17" s="0" t="str">
-        <f aca="false">IF(_xlfn.QUARTILE.INC(A2:A11, 3)&gt;7, "high", "low")</f>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.2">
+      <c r="G17" t="str">
+        <f>IF(_xlfn.QUARTILE.INC(A2:A11, 3)&gt;7, "high", "low")</f>
         <v>high</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G18" s="0" t="str">
-        <f aca="false">IFERROR(_xlfn.QUARTILE.EXC(A2:A11, 0), "n/a")</f>
+    <row r="18" spans="7:7" x14ac:dyDescent="0.2">
+      <c r="G18" t="str">
+        <f>IFERROR(_xlfn.QUARTILE.EXC(A2:A11, 0), "n/a")</f>
         <v>n/a</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G19" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(Sheet2!A2:A6, 2)</f>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.2">
+      <c r="G19">
+        <f>_xlfn.QUARTILE.INC(Sheet2!A2:A6, 2)</f>
         <v>30</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G20" s="0" t="n">
-        <f aca="false">_xlfn.QUARTILE.INC(A2:A11, 3) - _xlfn.QUARTILE.INC(A2:A11, 1)</f>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.2">
+      <c r="G20">
+        <f>_xlfn.QUARTILE.INC(A2:A11, 3) - _xlfn.QUARTILE.INC(A2:A11, 1)</f>
         <v>4.5</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>20</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>30</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>40</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>50</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>